<commit_message>
Fix of coverage logic
</commit_message>
<xml_diff>
--- a/data/testcases/Testcases.xlsx
+++ b/data/testcases/Testcases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahurt/Documents/DOCUMENTS/AI_COURSE/MY_WORK/QA_TEST_AGENT/data/testcases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B52CBE1-6640-0745-B3F2-FF51D69FF9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62466C86-6F5E-0340-BD4B-45421EA8F196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-45640" yWindow="1080" windowWidth="34360" windowHeight="20540" firstSheet="4" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-45640" yWindow="1080" windowWidth="34360" windowHeight="20540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Registration" sheetId="1" r:id="rId1"/>
@@ -9151,8 +9151,8 @@
     <col min="3" max="3" width="7.5" style="22" customWidth="1"/>
     <col min="4" max="4" width="51.6640625" style="23" customWidth="1"/>
     <col min="5" max="5" width="59.5" style="23" customWidth="1"/>
-    <col min="6" max="13" width="9.1640625" style="8" customWidth="1"/>
-    <col min="14" max="16384" width="9.1640625" style="8"/>
+    <col min="6" max="18" width="9.1640625" style="8" customWidth="1"/>
+    <col min="19" max="16384" width="9.1640625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="21" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
moved prompts to separate file, updated readme
</commit_message>
<xml_diff>
--- a/data/testcases/Testcases.xlsx
+++ b/data/testcases/Testcases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahurt/Documents/DOCUMENTS/AI_COURSE/MY_WORK/QA_TEST_AGENT/data/testcases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDE45D9F-4126-A248-A575-557110B373CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F27B7BC-35A7-854E-80E1-933DC9DF6646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-45640" yWindow="1080" windowWidth="34360" windowHeight="20540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9151,8 +9151,8 @@
     <col min="3" max="3" width="7.5" style="22" customWidth="1"/>
     <col min="4" max="4" width="51.6640625" style="23" customWidth="1"/>
     <col min="5" max="5" width="59.5" style="23" customWidth="1"/>
-    <col min="6" max="16" width="9.1640625" style="8" customWidth="1"/>
-    <col min="17" max="16384" width="9.1640625" style="8"/>
+    <col min="6" max="17" width="9.1640625" style="8" customWidth="1"/>
+    <col min="18" max="16384" width="9.1640625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="21" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
fix excel file - column for step number
</commit_message>
<xml_diff>
--- a/data/testcases/Testcases.xlsx
+++ b/data/testcases/Testcases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahurt/Documents/DOCUMENTS/AI_COURSE/MY_WORK/QA_TEST_AGENT/data/testcases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F27B7BC-35A7-854E-80E1-933DC9DF6646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E341DD47-829E-7F49-A6EA-B89BC28EF366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-45640" yWindow="1080" windowWidth="34360" windowHeight="20540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="200" yWindow="1020" windowWidth="34360" windowHeight="20540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Registration" sheetId="1" r:id="rId1"/>
@@ -9151,8 +9151,8 @@
     <col min="3" max="3" width="7.5" style="22" customWidth="1"/>
     <col min="4" max="4" width="51.6640625" style="23" customWidth="1"/>
     <col min="5" max="5" width="59.5" style="23" customWidth="1"/>
-    <col min="6" max="17" width="9.1640625" style="8" customWidth="1"/>
-    <col min="18" max="16384" width="9.1640625" style="8"/>
+    <col min="6" max="19" width="9.1640625" style="8" customWidth="1"/>
+    <col min="20" max="16384" width="9.1640625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="21" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -11166,7 +11166,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -11440,6 +11440,27 @@
       <c r="C22" s="93"/>
       <c r="D22" s="86"/>
       <c r="E22" s="94"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="18"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>